<commit_message>
Add copy-paste instruction page (Instructions tab + standalone .txt)
Clean usage guide: what it does, the tabs, 5-step add-a-deal, what
auto-calculates, verdict thresholds, the stress test, the reference models, and
a color key. Same text on the workbook's Instructions tab and as
IC_Dashboard_Instructions.txt for pasting into emails/decks.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016BmrADioxTa5RVaw6vVD9w
</commit_message>
<xml_diff>
--- a/ICGoNoGoDashboardDraftECAPJI.xlsx
+++ b/ICGoNoGoDashboardDraftECAPJI.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="170" formatCode="0_);\(0\)"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -159,8 +159,24 @@
       <i val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -242,6 +258,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A5F"/>
       </patternFill>
     </fill>
   </fills>
@@ -526,7 +547,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -891,6 +912,33 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1829,13 +1877,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="104" customWidth="1" style="151" min="1" max="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Instruction </t>
+    <row r="1" ht="26" customHeight="1" s="151">
+      <c r="A1" s="156" t="inlineStr">
+        <is>
+          <t>IC GO / NO-GO DASHBOARD — INSTRUCTIONS</t>
         </is>
       </c>
       <c r="B1" s="28" t="n"/>
@@ -1844,45 +1895,317 @@
       <c r="E1" s="29" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="n"/>
+      <c r="A2" s="157" t="inlineStr"/>
       <c r="E2" s="24" t="n"/>
     </row>
-    <row r="3">
-      <c r="A3" s="23" t="n"/>
+    <row r="3" ht="20" customHeight="1" s="151">
+      <c r="A3" s="158" t="inlineStr">
+        <is>
+          <t>WHAT IT DOES</t>
+        </is>
+      </c>
       <c r="E3" s="24" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
+      <c r="A4" s="159" t="inlineStr">
+        <is>
+          <t>Scores any deal GO / CONDITIONAL GO / NO-GO against four proven reference models and a</t>
+        </is>
+      </c>
       <c r="E4" s="24" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
+      <c r="A5" s="157" t="inlineStr">
+        <is>
+          <t>246-market ranking, with a downside stress test. Pick a deal and read the verdict.</t>
+        </is>
+      </c>
       <c r="E5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
+      <c r="A6" s="157" t="inlineStr"/>
       <c r="E6" s="24" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="23" t="n"/>
+    <row r="7" ht="20" customHeight="1" s="151">
+      <c r="A7" s="158" t="inlineStr">
+        <is>
+          <t>THE TABS</t>
+        </is>
+      </c>
       <c r="E7" s="24" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
+      <c r="A8" s="157" t="inlineStr">
+        <is>
+          <t>Dashboard ....... pick a deal in cell B3; see verdict, comparison vs the reference models,</t>
+        </is>
+      </c>
       <c r="E8" s="24" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
+      <c r="A9" s="157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 the gate scorecard, and the stress test.</t>
+        </is>
+      </c>
       <c r="E9" s="24" t="n"/>
     </row>
     <row r="10" ht="47.5" customHeight="1" s="151">
-      <c r="A10" s="25" t="n"/>
+      <c r="A10" s="160" t="inlineStr">
+        <is>
+          <t>Deals ........... every deal in a column. Yellow = you type · Blue = locked reference ·</t>
+        </is>
+      </c>
       <c r="B10" s="22" t="n"/>
       <c r="C10" s="22" t="n"/>
       <c r="D10" s="22" t="n"/>
       <c r="E10" s="26" t="n"/>
     </row>
-    <row r="11" ht="52" customHeight="1" s="151"/>
+    <row r="11" ht="52" customHeight="1" s="151">
+      <c r="A11" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 White = auto-calculated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="161" t="inlineStr">
+        <is>
+          <t>Cash Flows ...... annual equity cash flows per deal; =IRR computes the IRR below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="161" t="inlineStr">
+        <is>
+          <t>Scores .......... the live gate engine (one column per deal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="161" t="inlineStr">
+        <is>
+          <t>Ranking ......... all deals ranked by score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="161" t="inlineStr">
+        <is>
+          <t>Market Ranking / Market Data ... the 246-market data (Market Data is locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="161" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" s="151">
+      <c r="A17" s="162" t="inlineStr">
+        <is>
+          <t>HOW TO ADD A DEAL — 5 STEPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="163" t="inlineStr">
+        <is>
+          <t>1.  Deals tab: go to the first empty 'New Deal' column (yellow cells).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="163" t="inlineStr">
+        <is>
+          <t>2.  Pick the Deal type and the Market (county) from the dropdowns. Market data AND the</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     market's typical exit cap / yield / IRR / op-ex auto-fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="163" t="inlineStr">
+        <is>
+          <t>3.  Type the economics in the yellow cells: Total cost, Equity, Debt, Exit cap, NOI,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Op-ex ratio, Going-in cap (income deals), Unlevered IRR, Levered IRR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="163" t="inlineStr">
+        <is>
+          <t>4.  (Optional, for a true bottom-up IRR) Cash Flows tab: type the deal's annual equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     cash flows in its column (Year 0 = minus equity). =IRR computes automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="163" t="inlineStr">
+        <is>
+          <t>5.  Dashboard tab: pick the deal in cell B3 -&gt; read GO / CONDITIONAL GO / NO-GO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     the side-by-side vs the reference models, and the stress test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="161" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" s="151">
+      <c r="A28" s="162" t="inlineStr">
+        <is>
+          <t>WHAT AUTO-CALCULATES (do not type these)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="161" t="inlineStr">
+        <is>
+          <t>Is-development · LTV · Yield-on-cost · Dev spread · Equity IRR · Calculated IRR · every</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="161" t="inlineStr">
+        <is>
+          <t>market field (population, growth, pipeline, rank, and market exit cap / yield / IRR / op-ex).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="161" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" s="151">
+      <c r="A32" s="162" t="inlineStr">
+        <is>
+          <t>THE VERDICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="163" t="inlineStr">
+        <is>
+          <t>Score 70 or more = GO   ·   50 to 69 = CONDITIONAL GO   ·   under 50 = NO-GO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="161" t="inlineStr">
+        <is>
+          <t>Critical gates — failing ANY one forces NO-GO: IRR &gt; exit cap · yield at least 6.5% ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="161" t="inlineStr">
+        <is>
+          <t>market population at least 200,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="161" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" s="151">
+      <c r="A37" s="162" t="inlineStr">
+        <is>
+          <t>THE STRESS TEST (Dashboard, lower section)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="163" t="inlineStr">
+        <is>
+          <t>Applies exit cap +50 bps and NOI -5% to the selected deal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="161" t="inlineStr">
+        <is>
+          <t>'YES — robust' = the deal still works under stress.  'FRAGILE' = it fails under stress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="161" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="151">
+      <c r="A41" s="162" t="inlineStr">
+        <is>
+          <t>REFERENCE MODELS (blue, locked) — every deal is measured against these</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="161" t="inlineStr">
+        <is>
+          <t>Springfield (income / core) · Hamburg (storage development) ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="161" t="inlineStr">
+        <is>
+          <t>Dev 11-Mkt (workforce multifamily) · Factory Fund (operating company).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="161" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1" s="151">
+      <c r="A45" s="162" t="inlineStr">
+        <is>
+          <t>COLOR KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="161" t="inlineStr">
+        <is>
+          <t>Yellow = type here · Blue = locked reference / auto-pulled · White = formula ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="161" t="inlineStr">
+        <is>
+          <t>Green = gate passed · Red = gate failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="161" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="164" t="inlineStr">
+        <is>
+          <t>Not investment advice. Verify all figures independently.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>